<commit_message>
update DS with correction to instructions
</commit_message>
<xml_diff>
--- a/baseline/dataschema_ProPASS.xlsx
+++ b/baseline/dataschema_ProPASS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sbtiali\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F7C0088-3F20-40EB-9F16-7551435FB862}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E958CB-7E29-424A-8BB3-5E8E4A3DEEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{DB9EE49B-F8BF-4815-B441-B0BA94DBFC22}"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2275" uniqueCount="570">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2277" uniqueCount="572">
   <si>
     <t>index</t>
   </si>
@@ -1796,6 +1796,12 @@
   </si>
   <si>
     <t>Crosscheck with dis_diabetes_ever.</t>
+  </si>
+  <si>
+    <t>If one or two values are missing from the score, then they can be substituted with the average score of the non-missing items. Questionnaires with more than two missing values should be disregarded.</t>
+  </si>
+  <si>
+    <t>Includes osteoporosis, arthrosis, rheumatic disorder, osteoarthritis or rheumatism, rheumatoid arthritis, osteoarthritis, other arthritis, rheumatoid arthritis.</t>
   </si>
 </sst>
 </file>
@@ -1851,7 +1857,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2168,9 +2174,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F8E0180-A72F-4AF4-960B-1515820225EB}">
   <dimension ref="A1:P122"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="11.42578125" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="4" max="4" width="35.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -5451,6 +5458,9 @@
       <c r="L87" t="s">
         <v>46</v>
       </c>
+      <c r="M87" t="s">
+        <v>571</v>
+      </c>
       <c r="N87" t="s">
         <v>372</v>
       </c>
@@ -6405,7 +6415,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>112</v>
       </c>
@@ -6440,7 +6450,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>113</v>
       </c>
@@ -6475,7 +6485,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>114</v>
       </c>
@@ -6510,7 +6520,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>115</v>
       </c>
@@ -6545,7 +6555,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>116</v>
       </c>
@@ -6580,7 +6590,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>117</v>
       </c>
@@ -6615,7 +6625,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>118</v>
       </c>
@@ -6650,7 +6660,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>119</v>
       </c>
@@ -6684,8 +6694,11 @@
       <c r="N120" t="s">
         <v>481</v>
       </c>
-    </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="O120" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>120</v>
       </c>
@@ -6720,7 +6733,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>121</v>
       </c>
@@ -6763,7 +6776,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D6186D5-BB84-4E3C-AAC4-F17A4EDF9A5A}">
   <dimension ref="A1:F237"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" bestFit="1" customWidth="1"/>

</xml_diff>